<commit_message>
v2.0.3: Codex-Findings - Auslagen-Konsistenz, Akteninhalt-Typo, Anlagen-Beispiel ASCII
Drei Findings von Codex aufgenommen:

1. testakten/fluggastrechte-familie-braeutigam/Aufstellung_Auslagen.xlsx:
   G34-G37 waren mit gerundeten Werten (387/110/48/27) hartcodiert, sodass
   GESAMTFORDERUNG (G40) 3572 EUR auswarf - waehrend die Auslagen-Tabelle
   intern 587,64 EUR rechnete. G34-G37 jetzt als =G25..=G28 verformelt,
   Excel ist nun in sich konsistent (G30 = G34+G35+G36+G37 = 587,64;
   G40 = 3587,64).

2. README der Fluggastrechte-Testakte: 'ca. 545 EUR' / 'ca. 3.545 EUR' an
   die Excel-Werte 587,64 / 3.587,64 angeglichen. Typo 'Akteiinhalt' ->
   'Akteninhalt'. H33-Bemerkung der Excel C-257/14 -> C-549/07 nachgezogen.

3. anlagen-zu-schriftsaetzen/SKILL.md: Beispiel 'Aufrechnungserklaerung'
   ASCII-fiziert. Vorher widersprach 'Anlage_B-01_Aufrechnungserklaerung.pdf'
   mit Umlaut direkt der drei Zeilen darunter stehenden Regel 'Keine Umlaute,
   kein scharfes ss'.
</commit_message>
<xml_diff>
--- a/testakten/fluggastrechte-familie-braeutigam/Aufstellung_Auslagen.xlsx
+++ b/testakten/fluggastrechte-familie-braeutigam/Aufstellung_Auslagen.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00 &quot;EUR&quot;"/>
+  </numFmts>
   <fonts count="19">
     <font>
       <name val="Calibri"/>
@@ -258,7 +260,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -383,6 +385,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1633,12 +1647,12 @@
       </c>
       <c r="E33" s="25" t="n"/>
       <c r="F33" s="25" t="n"/>
-      <c r="G33" s="33" t="n">
+      <c r="G33" s="47" t="n">
         <v>3000</v>
       </c>
       <c r="H33" s="34" t="inlineStr">
         <is>
-          <t>VO (EG) 261/2004 Art. 7 (1)(c): &gt;3.500 km (8.954 km BKK-FRA), Verspätung 53h (&gt;4h), techn. Problem kein auß. Umstand (EuGH C-257/14)</t>
+          <t>VO (EG) 261/2004 Art. 7 (1)(c): &gt;3.500 km (8.954 km BKK-FRA), Verspätung 53h (&gt;4h), techn. Problem kein auß. Umstand (EuGH C-549/07)</t>
         </is>
       </c>
       <c r="I33" s="35" t="n"/>
@@ -1658,8 +1672,9 @@
       </c>
       <c r="E34" s="38" t="n"/>
       <c r="F34" s="38" t="n"/>
-      <c r="G34" s="40" t="n">
-        <v>387</v>
+      <c r="G34" s="48">
+        <f>G25</f>
+        <v/>
       </c>
       <c r="H34" s="41" t="inlineStr">
         <is>
@@ -1683,8 +1698,9 @@
       </c>
       <c r="E35" s="25" t="n"/>
       <c r="F35" s="25" t="n"/>
-      <c r="G35" s="33" t="n">
-        <v>110</v>
+      <c r="G35" s="47">
+        <f>G26</f>
+        <v/>
       </c>
       <c r="H35" s="34" t="inlineStr">
         <is>
@@ -1708,8 +1724,9 @@
       </c>
       <c r="E36" s="38" t="n"/>
       <c r="F36" s="38" t="n"/>
-      <c r="G36" s="40" t="n">
-        <v>48</v>
+      <c r="G36" s="48">
+        <f>G27</f>
+        <v/>
       </c>
       <c r="H36" s="41" t="inlineStr">
         <is>
@@ -1733,8 +1750,9 @@
       </c>
       <c r="E37" s="25" t="n"/>
       <c r="F37" s="25" t="n"/>
-      <c r="G37" s="33" t="n">
-        <v>27</v>
+      <c r="G37" s="47">
+        <f>G28</f>
+        <v/>
       </c>
       <c r="H37" s="34" t="inlineStr">
         <is>
@@ -1758,7 +1776,7 @@
       </c>
       <c r="E38" s="38" t="n"/>
       <c r="F38" s="38" t="n"/>
-      <c r="G38" s="42" t="n">
+      <c r="G38" s="49" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="41" t="inlineStr">
@@ -1779,7 +1797,7 @@
       <c r="D40" s="44" t="n"/>
       <c r="E40" s="44" t="n"/>
       <c r="F40" s="44" t="n"/>
-      <c r="G40" s="45">
+      <c r="G40" s="50">
         <f>SUM(G33:G38)</f>
         <v/>
       </c>

</xml_diff>